<commit_message>
feat(pa): asignacion por area, aceptacion docente y catalogo importable
</commit_message>
<xml_diff>
--- a/esap/programacion/resultados/2026-1/catalogo-conciliacion.xlsx
+++ b/esap/programacion/resultados/2026-1/catalogo-conciliacion.xlsx
@@ -4,7 +4,8 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="CONCILIACION_NO_IMPORTAR" sheetId="1" r:id="rId1"/>
-    <sheet name="LEEME" sheetId="2" r:id="rId2"/>
+    <sheet name="REVISION_MANUAL" sheetId="2" r:id="rId2"/>
+    <sheet name="LEEME" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -18977,6 +18978,102 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>fila_programacion</v>
+      </c>
+      <c r="B1" t="str">
+        <v>plan</v>
+      </c>
+      <c r="C1" t="str">
+        <v>asignatura_programada</v>
+      </c>
+      <c r="D1" t="str">
+        <v>candidatos_plan</v>
+      </c>
+      <c r="E1" t="str">
+        <v>decision</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fila-35</v>
+      </c>
+      <c r="B2" t="str">
+        <v>APT_52</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Opción de grado</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Opción de grado (Curso Profundización temática 1) | Opción de grado (Curso Profundización temática 2)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>REVISAR A MANO: no hay coincidencia exacta; no se asigna código ni se fusionan asignaturas</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fila-36</v>
+      </c>
+      <c r="B3" t="str">
+        <v>APT_52</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Opción de grado</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Opción de grado (Curso Profundización temática 1) | Opción de grado (Curso Profundización temática 2)</v>
+      </c>
+      <c r="E3" t="str">
+        <v>REVISAR A MANO: no hay coincidencia exacta; no se asigna código ni se fusionan asignaturas</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fila-440</v>
+      </c>
+      <c r="B4" t="str">
+        <v>APT_52</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Opción de grado</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Opción de grado (Curso Profundización temática 1) | Opción de grado (Curso Profundización temática 2)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>REVISAR A MANO: no hay coincidencia exacta; no se asigna código ni se fusionan asignaturas</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>fila-441</v>
+      </c>
+      <c r="B5" t="str">
+        <v>APT_52</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Opción de grado</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Opción de grado (Curso Profundización temática 1) | Opción de grado (Curso Profundización temática 2)</v>
+      </c>
+      <c r="E5" t="str">
+        <v>REVISAR A MANO: no hay coincidencia exacta; no se asigna código ni se fusionan asignaturas</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
feat(pa): persist subject area decisions and measure additive bridge coverage
</commit_message>
<xml_diff>
--- a/esap/programacion/resultados/2026-1/catalogo-conciliacion.xlsx
+++ b/esap/programacion/resultados/2026-1/catalogo-conciliacion.xlsx
@@ -2897,10 +2897,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K57" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L57" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M57">
         <v>15</v>
@@ -2982,7 +2982,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J59" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K59" t="str">
         <v>NT-013</v>
@@ -3073,10 +3073,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K61" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L61" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M61">
         <v>3</v>
@@ -3205,10 +3205,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K64" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L64" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M64">
         <v>3</v>
@@ -3246,7 +3246,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J65" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K65" t="str">
         <v>NT-013</v>
@@ -3284,7 +3284,7 @@
         <v>0</v>
       </c>
       <c r="H66" t="str">
-        <v>ASIG-00177 (PRO-003, pensum sin definir) | ASIG-00182 (PRO-003, pensum sin definir)</v>
+        <v>ASIG-00182 (PRO-003, pensum sin definir) | ASIG-00177 (PRO-003, pensum sin definir)</v>
       </c>
       <c r="I66" t="str">
         <v>Organizaciones públicas</v>
@@ -3469,10 +3469,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K70" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L70" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M70">
         <v>3</v>
@@ -3510,7 +3510,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J71" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K71" t="str">
         <v>NT-013</v>
@@ -3686,7 +3686,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J75" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K75" t="str">
         <v>NT-013</v>
@@ -3730,7 +3730,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J76" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K76" t="str">
         <v>NT-013</v>
@@ -4129,10 +4129,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K85" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L85" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M85">
         <v>3</v>
@@ -4173,10 +4173,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K86" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L86" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M86">
         <v>4</v>
@@ -4393,10 +4393,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K91" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L91" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M91">
         <v>4</v>
@@ -4434,7 +4434,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J92" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K92" t="str">
         <v>NT-013</v>
@@ -4613,10 +4613,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K96" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L96" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M96">
         <v>3</v>
@@ -4833,10 +4833,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K101" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L101" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M101">
         <v>4</v>
@@ -5097,10 +5097,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K107" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L107" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M107">
         <v>7</v>
@@ -7561,10 +7561,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K163" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L163" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M163">
         <v>15</v>
@@ -7781,10 +7781,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K168" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L168" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M168">
         <v>3</v>
@@ -7913,10 +7913,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K171" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L171" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M171">
         <v>3</v>
@@ -7954,7 +7954,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J172" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K172" t="str">
         <v>NT-013</v>
@@ -7992,7 +7992,7 @@
         <v>0</v>
       </c>
       <c r="H173" t="str">
-        <v>ASIG-00177 (PRO-003, pensum sin definir) | ASIG-00182 (PRO-003, pensum sin definir)</v>
+        <v>ASIG-00182 (PRO-003, pensum sin definir) | ASIG-00177 (PRO-003, pensum sin definir)</v>
       </c>
       <c r="I173" t="str">
         <v>Organizaciones públicas</v>
@@ -8133,10 +8133,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K176" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L176" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M176">
         <v>3</v>
@@ -8174,7 +8174,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J177" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K177" t="str">
         <v>NT-013</v>
@@ -8350,7 +8350,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J181" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K181" t="str">
         <v>NT-013</v>
@@ -8438,7 +8438,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J183" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K183" t="str">
         <v>NT-013</v>
@@ -8790,7 +8790,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J191" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K191" t="str">
         <v>NT-013</v>
@@ -9013,10 +9013,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K196" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L196" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M196">
         <v>3</v>
@@ -9057,10 +9057,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K197" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L197" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M197">
         <v>4</v>
@@ -9101,10 +9101,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K198" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L198" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M198">
         <v>3</v>
@@ -9230,7 +9230,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J201" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K201" t="str">
         <v>NT-013</v>
@@ -9453,10 +9453,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K206" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L206" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M206">
         <v>4</v>
@@ -9673,10 +9673,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K211" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L211" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M211">
         <v>3</v>
@@ -9717,10 +9717,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K212" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L212" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M212">
         <v>4</v>
@@ -10808,7 +10808,7 @@
         <v>0</v>
       </c>
       <c r="H237" t="str">
-        <v>ASIG-00177 (PRO-003, pensum sin definir) | ASIG-00182 (PRO-003, pensum sin definir)</v>
+        <v>ASIG-00182 (PRO-003, pensum sin definir) | ASIG-00177 (PRO-003, pensum sin definir)</v>
       </c>
       <c r="I237" t="str">
         <v>Problemática del Estado y del Poder</v>
@@ -11257,10 +11257,10 @@
         <v>Finanzas Públicas</v>
       </c>
       <c r="K247" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="L247" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M247">
         <v>3</v>
@@ -12357,10 +12357,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K272" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L272" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M272">
         <v>4</v>
@@ -12401,10 +12401,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K273" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L273" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M273">
         <v>4</v>
@@ -12445,10 +12445,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K274" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L274" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M274">
         <v>4</v>
@@ -12489,10 +12489,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K275" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L275" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M275">
         <v>4</v>
@@ -12618,7 +12618,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J278" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K278" t="str">
         <v>NT-013</v>
@@ -12662,7 +12662,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J279" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K279" t="str">
         <v>NT-013</v>
@@ -12882,7 +12882,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J284" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K284" t="str">
         <v>NT-013</v>
@@ -12926,7 +12926,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J285" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K285" t="str">
         <v>NT-013</v>
@@ -13140,13 +13140,13 @@
         <v>0</v>
       </c>
       <c r="H290" t="str">
-        <v>ASIG-00177 (PRO-003, pensum sin definir) | ASIG-00182 (PRO-003, pensum sin definir)</v>
+        <v>ASIG-00182 (PRO-003, pensum sin definir) | ASIG-00177 (PRO-003, pensum sin definir)</v>
       </c>
       <c r="I290" t="str">
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J290" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K290" t="str">
         <v>NT-013</v>
@@ -13190,7 +13190,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J291" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K291" t="str">
         <v>NT-013</v>
@@ -13410,7 +13410,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J296" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K296" t="str">
         <v>NT-013</v>
@@ -13454,7 +13454,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J297" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K297" t="str">
         <v>NT-013</v>
@@ -13498,7 +13498,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J298" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K298" t="str">
         <v>NT-013</v>
@@ -13718,7 +13718,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J303" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K303" t="str">
         <v>NT-013</v>
@@ -13938,7 +13938,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J308" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K308" t="str">
         <v>NT-013</v>
@@ -13982,7 +13982,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J309" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K309" t="str">
         <v>NT-013</v>
@@ -14246,7 +14246,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J315" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K315" t="str">
         <v>NT-013</v>
@@ -14466,7 +14466,7 @@
         <v>Estado Gobierno y Sociedad</v>
       </c>
       <c r="J320" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
+        <v>Estado y Poder</v>
       </c>
       <c r="K320" t="str">
         <v>NT-013</v>
@@ -14645,10 +14645,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K324" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L324" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M324">
         <v>6</v>
@@ -14821,10 +14821,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K328" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L328" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M328">
         <v>3</v>
@@ -14865,10 +14865,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K329" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L329" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M329">
         <v>3</v>
@@ -16977,10 +16977,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K377" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L377" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M377">
         <v>10</v>
@@ -18957,10 +18957,10 @@
         <v>Opción de grado</v>
       </c>
       <c r="K422" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="L422" t="str">
-        <v>Área sin código único: revisar</v>
+        <v>Sin coincidencia exacta: revisar antes de crear</v>
       </c>
       <c r="M422">
         <v>10</v>

</xml_diff>